<commit_message>
Improve user deactivate/update: add logging
Add input validation, logging and stronger DynamoDB operations for user deactivation/update. deactivate_user.py: add logger, require USERS_TABLE_NAME, default REGION, robust body parsing, validate_user_id helper, switch to update_item with ConditionExpression (raises ValueError if user missing), and improved error handling/response codes. update_user.py: set default REGION and tighten ConditionExpression to require ACTIVE=True when updating. Also add test notebooks for create/deactivate/update lambdas and update backend/aws/info.xlsx binary.
</commit_message>
<xml_diff>
--- a/backend/aws/info.xlsx
+++ b/backend/aws/info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucia\Documents\GitHub\TFG_Posdata\backend\aws\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B73687B-4E17-4573-9BCC-2128429CB66E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B90CD507-6FD8-4851-B5DC-C4E59DD2D7ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{717247B1-5BD0-4CA7-8E56-C22B8892B153}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>AWS Service</t>
   </si>
@@ -96,6 +96,13 @@
   <si>
     <t>Handles dynamic user updates in DynamoDB. Performs schema validation for 
 emergency contacts and accessibility settings, using Attribute Name Aliasing to prevent reserved word collisions and ensuring record existence via Condition Expressions.</t>
+  </si>
+  <si>
+    <t>Handles soft deletion of user accounts in DynamoDB. Validates input identifiers 
+and performs a partial update to set the ACTIVE flag to false. Includes conditional logic to fail gracefully if the targeted User ID is not found in the database.</t>
+  </si>
+  <si>
+    <t>Test cases</t>
   </si>
 </sst>
 </file>
@@ -221,7 +228,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -238,24 +245,27 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -265,8 +275,8 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -582,16 +592,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC3E1799-8E9C-484C-98AD-CB385F3A2068}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.26953125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="37.08984375" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="70.08984375" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="70.90625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="15" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -604,96 +614,101 @@
       <c r="D1" s="5" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
+      <c r="E1" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="6"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="8" t="s">
+    <row r="3" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="11"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="6"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="8" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="11"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="10"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="6"/>
-      <c r="B5" s="7" t="s">
+      <c r="D4" s="9"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="11"/>
+      <c r="B5" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="10"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="6"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="8" t="s">
+      <c r="D5" s="9"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="11"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="10"/>
-    </row>
-    <row r="7" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="6"/>
-      <c r="B7" s="12" t="s">
+      <c r="D6" s="9"/>
+    </row>
+    <row r="7" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="11"/>
+      <c r="B7" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A8" s="6"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="8" t="s">
+    <row r="8" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A8" s="11"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="6"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="8" t="s">
+    <row r="9" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="11"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="10"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="6"/>
-      <c r="B10" s="11" t="s">
+      <c r="D9" s="16" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="11"/>
+      <c r="B10" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="10"/>
+      <c r="D10" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Enhance CSV-to-DynamoDB Lambda with logging
Update insert_items_into_dynamodb.py to improve robustness and observability: add logging and json imports, validate required env var LISTS_TABLE_NAME and set a default REGION_NAME, stream CSV directly from S3, validate rows contain PK/SK/DESCRIPTION, add UPLOAD_DATE, use batch_writer with a processed count, handle multiple S3 Records, skip non-CSV files, and surface ClientError/internal errors with structured responses. Also update backend/aws/info.xlsx (binary change). These changes make the Lambda safer for production and easier to debug.
</commit_message>
<xml_diff>
--- a/backend/aws/info.xlsx
+++ b/backend/aws/info.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucia\Documents\GitHub\TFG_Posdata\backend\aws\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B90CD507-6FD8-4851-B5DC-C4E59DD2D7ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33C00105-3563-4389-9A82-C275E7B4E462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{717247B1-5BD0-4CA7-8E56-C22B8892B153}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{717247B1-5BD0-4CA7-8E56-C22B8892B153}"/>
   </bookViews>
   <sheets>
-    <sheet name="Lambda" sheetId="1" r:id="rId1"/>
+    <sheet name="DynamoDB" sheetId="2" r:id="rId1"/>
+    <sheet name="Lambda" sheetId="1" r:id="rId2"/>
+    <sheet name="S3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="48">
   <si>
     <t>AWS Service</t>
   </si>
@@ -37,9 +39,6 @@
   </si>
   <si>
     <t>Lambda</t>
-  </si>
-  <si>
-    <t>posdata-listssmschech-lambda</t>
   </si>
   <si>
     <t>SMS Verdict Engine: Performs multi-stage validation of incoming messages against
@@ -102,7 +101,83 @@
 and performs a partial update to set the ACTIVE flag to false. Includes conditional logic to fail gracefully if the targeted User ID is not found in the database.</t>
   </si>
   <si>
-    <t>Test cases</t>
+    <t>Automates CSV data ingestion from S3 to DynamoDB. Includes memory-optimized 
+streaming, schema validation, and high-throughput batch writing to ensure efficient data migration and synchronization."</t>
+  </si>
+  <si>
+    <t>Python 3.14</t>
+  </si>
+  <si>
+    <t>Layers</t>
+  </si>
+  <si>
+    <t>posdata-utils-layer v8</t>
+  </si>
+  <si>
+    <t>Trigger</t>
+  </si>
+  <si>
+    <t>Destination</t>
+  </si>
+  <si>
+    <t>posdata-listssmscheck-lambda</t>
+  </si>
+  <si>
+    <t>posdata-hashlearning-queue</t>
+  </si>
+  <si>
+    <t>posdata-smslists-s3</t>
+  </si>
+  <si>
+    <t>Language Version</t>
+  </si>
+  <si>
+    <t>posdata-smslists-db</t>
+  </si>
+  <si>
+    <t>posdata-users-db</t>
+  </si>
+  <si>
+    <t>DynamoDB</t>
+  </si>
+  <si>
+    <t>SMS - Lists update</t>
+  </si>
+  <si>
+    <t>Partition Key</t>
+  </si>
+  <si>
+    <t>Sort Key</t>
+  </si>
+  <si>
+    <t>PK (String)</t>
+  </si>
+  <si>
+    <t>SK (String)</t>
+  </si>
+  <si>
+    <t>ARN</t>
+  </si>
+  <si>
+    <t>arn:aws:dynamodb:eu-west-3:170722810141:table/posdata-smslists-db</t>
+  </si>
+  <si>
+    <t>arn:aws:dynamodb:eu-west-3:170722810141:table/posdata-users-db</t>
+  </si>
+  <si>
+    <t>arn:aws:lambda:eu-west-3:170722810141:function:posdata-updateuser-lambda</t>
+  </si>
+  <si>
+    <t>arn:aws:lambda:eu-west-3:170722810141:function:posdata-listssmscheck-lambda</t>
+  </si>
+  <si>
+    <t>arn:aws:lambda:eu-west-3:170722810141:function:posdata-insertitemsintodynamodb-lambda</t>
+  </si>
+  <si>
+    <t>arn:aws:lambda:eu-west-3:170722810141:function:posdata-deactivate-user</t>
+  </si>
+  <si>
+    <t>arn:aws:lambda:eu-west-3:170722810141:function:posdata-learnhash-lambda</t>
   </si>
 </sst>
 </file>
@@ -126,7 +201,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -163,8 +238,44 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCCFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -208,17 +319,6 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -228,7 +328,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -260,23 +360,56 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -284,6 +417,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFCCFF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -591,124 +729,338 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AAE0A43-D9F4-4772-8EF4-455A5F157D98}">
+  <sheetPr>
+    <tabColor theme="4"/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.90625" style="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.54296875" style="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="61.36328125" style="19" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="20"/>
+      <c r="B3" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="21"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="20"/>
+      <c r="B4" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="23"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="20"/>
+      <c r="B5" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="21"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="23"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D4:D5"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC3E1799-8E9C-484C-98AD-CB385F3A2068}">
-  <dimension ref="A1:E10"/>
+  <sheetPr>
+    <tabColor theme="5"/>
+  </sheetPr>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.26953125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="37.08984375" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="70.90625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="83.36328125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="70.90625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="F1" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="15" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="12" t="s">
+      <c r="G2" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+    </row>
+    <row r="3" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="12"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="I3" s="16"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="12"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="11"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="8" t="s">
+      <c r="D4" s="7"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="12"/>
+      <c r="B5" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="7"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="12"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="7"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+    </row>
+    <row r="7" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="12"/>
+      <c r="B7" s="13" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="11"/>
-      <c r="B4" s="12"/>
-      <c r="C4" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="9"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="11"/>
-      <c r="B5" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="9"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="11"/>
-      <c r="B6" s="12"/>
-      <c r="C6" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="9"/>
-    </row>
-    <row r="7" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="11"/>
-      <c r="B7" s="13" t="s">
+      <c r="C7" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+    </row>
+    <row r="8" spans="1:9" ht="58" x14ac:dyDescent="0.35">
+      <c r="A8" s="12"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G8" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="16"/>
+      <c r="I8" s="16"/>
+    </row>
+    <row r="9" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="12"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G9" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+    </row>
+    <row r="10" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="12"/>
+      <c r="B10" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="58" x14ac:dyDescent="0.35">
-      <c r="A8" s="11"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="11"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="7" t="s">
+      <c r="C10" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D10" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="14" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="11"/>
-      <c r="B10" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="9"/>
+      <c r="F10" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G10" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -719,4 +1071,16 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1FCA5BB-BB75-4692-B0DF-C8BE087A85D5}">
+  <sheetPr>
+    <tabColor theme="9"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>